<commit_message>
Valutazioni: ricerca OMI anche fuori Treviso, con comune dall'Excel o dall'indirizzo e provincia automatica
- comune dalla pagina, dalla nuova cella COMUNE dell'Excel o dall'indirizzo ("Via Roma 10, Jesolo"),
  altrimenti quello predefinito; la provincia si ricava dal comune (elenco ISTAT dei comuni)
- avvisi se la provincia scritta non corrisponde al comune o il comune non esiste
- nella pagina si vede quale comune si cerca e da dove viene; nel Word il nome ufficiale del comune

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GFqWfsVatsLJvctcKSGrA2
</commit_message>
<xml_diff>
--- a/valutazioni/modelli/stima_modello.xlsx
+++ b/valutazioni/modelli/stima_modello.xlsx
@@ -303,7 +303,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -432,6 +432,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -513,11 +514,17 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Valutazioni</author>
+    <author>Grigolo</author>
   </authors>
   <commentList>
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
         <t>Zona OMI in cui si trova l'immobile: il codice (es. B1) oppure il nome della zona come compare sul sito dell'Agenzia delle Entrate (es. Centro storico).</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="1" shapeId="0">
+      <text>
+        <t>Comune dell'immobile (es. Jesolo): serve per cercare i valori OMI. La provincia si ricava da sola. Se vuoto si usa il comune scritto nell'indirizzo, altrimenti quello predefinito (Treviso).</t>
       </text>
     </comment>
     <comment ref="F6" authorId="0" shapeId="0">
@@ -858,6 +865,12 @@
         </is>
       </c>
       <c r="B5" s="33" t="n"/>
+      <c r="C5" s="44" t="inlineStr">
+        <is>
+          <t>COMUNE:</t>
+        </is>
+      </c>
+      <c r="D5" s="62" t="n"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>DATA:</t>
@@ -1340,8 +1353,8 @@
     <mergeCell ref="C43:D43"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="C46:D46"/>
+    <mergeCell ref="F6:H6"/>
     <mergeCell ref="C38:D38"/>
-    <mergeCell ref="F6:H6"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="A42:B42"/>
     <mergeCell ref="C37:D37"/>

</xml_diff>